<commit_message>
continue lamatole adhuro bhawan thekka
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/thekka/लामाटोल अधुरो भवन/लामाटोल अधुरो भवन.xlsx
+++ b/बजेट माग estimate/thekka/लामाटोल अधुरो भवन/लामाटोल अधुरो भवन.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF2CF79-D992-4D24-A7C8-70ABBCADBBE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4E7945-B7B8-4FDC-8636-4AEAD1BE5F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -669,7 +669,7 @@
     <t>Grand total</t>
   </si>
   <si>
-    <t>-MS square pipe for post of 3"*75mm*5mm thickness</t>
+    <t>-MS square pipe for post of 3" * 3" * 2mm thickness</t>
   </si>
 </sst>
 </file>
@@ -995,6 +995,24 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1010,24 +1028,6 @@
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1573,113 +1573,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64"/>
-      <c r="K5" s="64"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="60"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="66" t="s">
+      <c r="H6" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="66"/>
-      <c r="J6" s="66"/>
-      <c r="K6" s="66"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="56" t="s">
+      <c r="H7" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
@@ -4982,11 +4982,11 @@
       <c r="B153" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="C153" s="57">
+      <c r="C153" s="63">
         <f>J151</f>
         <v>520268.58119831659</v>
       </c>
-      <c r="D153" s="58"/>
+      <c r="D153" s="64"/>
       <c r="E153" s="39">
         <v>100</v>
       </c>
@@ -5001,21 +5001,21 @@
       <c r="B154" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="C154" s="59">
+      <c r="C154" s="65">
         <v>700000</v>
       </c>
-      <c r="D154" s="60"/>
+      <c r="D154" s="66"/>
       <c r="E154" s="39"/>
     </row>
     <row r="155" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B155" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C155" s="59">
+      <c r="C155" s="65">
         <f>C154-C157-C158</f>
         <v>665000</v>
       </c>
-      <c r="D155" s="60"/>
+      <c r="D155" s="66"/>
       <c r="E155" s="39">
         <f>C155/C153*100</f>
         <v>127.81859678482381</v>
@@ -5039,11 +5039,11 @@
       <c r="B157" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="C157" s="57">
+      <c r="C157" s="63">
         <f>C154*0.03</f>
         <v>21000</v>
       </c>
-      <c r="D157" s="58"/>
+      <c r="D157" s="64"/>
       <c r="E157" s="39">
         <v>3</v>
       </c>
@@ -5052,17 +5052,23 @@
       <c r="B158" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C158" s="57">
+      <c r="C158" s="63">
         <f>C154*0.02</f>
         <v>14000</v>
       </c>
-      <c r="D158" s="58"/>
+      <c r="D158" s="64"/>
       <c r="E158" s="39">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C158:D158"/>
+    <mergeCell ref="C153:D153"/>
+    <mergeCell ref="C154:D154"/>
+    <mergeCell ref="C155:D155"/>
+    <mergeCell ref="C156:D156"/>
+    <mergeCell ref="C157:D157"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="H7:K7"/>
     <mergeCell ref="A1:K1"/>
@@ -5072,12 +5078,6 @@
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
-    <mergeCell ref="C158:D158"/>
-    <mergeCell ref="C153:D153"/>
-    <mergeCell ref="C154:D154"/>
-    <mergeCell ref="C155:D155"/>
-    <mergeCell ref="C156:D156"/>
-    <mergeCell ref="C157:D157"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="portrait" r:id="rId1"/>
@@ -5104,113 +5104,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64"/>
-      <c r="K5" s="64"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="60"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="55" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="66" t="s">
+      <c r="H6" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="66"/>
-      <c r="J6" s="66"/>
-      <c r="K6" s="66"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="56" t="s">
+      <c r="H7" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
@@ -7161,11 +7161,11 @@
       <c r="B99" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="C99" s="57">
+      <c r="C99" s="63">
         <f>J97</f>
         <v>1449733.6784769716</v>
       </c>
-      <c r="D99" s="58"/>
+      <c r="D99" s="64"/>
       <c r="E99" s="39">
         <v>100</v>
       </c>
@@ -7181,10 +7181,10 @@
       <c r="B100" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="C100" s="59">
+      <c r="C100" s="65">
         <v>1600000</v>
       </c>
-      <c r="D100" s="60"/>
+      <c r="D100" s="66"/>
       <c r="E100" s="39"/>
     </row>
     <row r="101" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -7192,11 +7192,11 @@
       <c r="B101" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C101" s="59">
+      <c r="C101" s="65">
         <f>C100-C103-C104</f>
         <v>1520000</v>
       </c>
-      <c r="D101" s="60"/>
+      <c r="D101" s="66"/>
       <c r="E101" s="39">
         <f>C101/C99*100</f>
         <v>104.84684342829418</v>
@@ -7222,11 +7222,11 @@
       <c r="B103" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="C103" s="57">
+      <c r="C103" s="63">
         <f>C100*0.03</f>
         <v>48000</v>
       </c>
-      <c r="D103" s="58"/>
+      <c r="D103" s="64"/>
       <c r="E103" s="39">
         <v>3</v>
       </c>
@@ -7236,24 +7236,17 @@
       <c r="B104" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C104" s="57">
+      <c r="C104" s="63">
         <f>C100*0.02</f>
         <v>32000</v>
       </c>
-      <c r="D104" s="58"/>
+      <c r="D104" s="64"/>
       <c r="E104" s="39">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C103:D103"/>
     <mergeCell ref="C104:D104"/>
     <mergeCell ref="A7:F7"/>
@@ -7262,6 +7255,13 @@
     <mergeCell ref="C100:D100"/>
     <mergeCell ref="C101:D101"/>
     <mergeCell ref="C102:D102"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="portrait" r:id="rId1"/>
@@ -7288,113 +7288,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64"/>
-      <c r="K5" s="64"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="60"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="55" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="66" t="s">
+      <c r="H6" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="66"/>
-      <c r="J6" s="66"/>
-      <c r="K6" s="66"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="56" t="s">
+      <c r="H7" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
@@ -7984,15 +7984,15 @@
         <v>0.3</v>
       </c>
       <c r="E33" s="3">
-        <v>10.5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="F33" s="3">
         <f>PRODUCT(C33:E33)</f>
-        <v>94.5</v>
+        <v>39.6</v>
       </c>
       <c r="G33" s="3">
         <f>F33</f>
-        <v>94.5</v>
+        <v>39.6</v>
       </c>
       <c r="H33" s="15"/>
       <c r="I33" s="15"/>
@@ -8009,15 +8009,15 @@
         <v>0.3</v>
       </c>
       <c r="E34" s="3">
-        <v>10.5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="F34" s="3">
         <f>PRODUCT(C34:E34)</f>
-        <v>103.95</v>
+        <v>43.56</v>
       </c>
       <c r="G34" s="3">
         <f>F34</f>
-        <v>103.95</v>
+        <v>43.56</v>
       </c>
       <c r="H34" s="15"/>
       <c r="I34" s="15"/>
@@ -8197,7 +8197,7 @@
       <c r="F41" s="20"/>
       <c r="G41" s="2">
         <f>SUM(G33:G40)</f>
-        <v>940.02269125266685</v>
+        <v>824.73269125266677</v>
       </c>
       <c r="H41" s="21" t="s">
         <v>108</v>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J41" s="22">
         <f>G41*I41</f>
-        <v>197298.07258760286</v>
+        <v>173100.25800260284</v>
       </c>
       <c r="K41" s="20"/>
     </row>
@@ -8323,7 +8323,7 @@
       <c r="I47" s="22"/>
       <c r="J47" s="22">
         <f>SUM(J13:J45)</f>
-        <v>405100.11710102775</v>
+        <v>380902.30251602776</v>
       </c>
       <c r="K47" s="36"/>
     </row>
@@ -8335,11 +8335,11 @@
       <c r="B49" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="C49" s="57">
+      <c r="C49" s="63">
         <f>J47</f>
-        <v>405100.11710102775</v>
-      </c>
-      <c r="D49" s="58"/>
+        <v>380902.30251602776</v>
+      </c>
+      <c r="D49" s="64"/>
       <c r="E49" s="37"/>
       <c r="F49" s="40"/>
       <c r="G49" s="37"/>
@@ -8352,25 +8352,30 @@
       <c r="B50" s="54" t="s">
         <v>128</v>
       </c>
-      <c r="C50" s="59">
+      <c r="C50" s="65">
         <f>0.13*C49</f>
-        <v>52663.015223133611</v>
-      </c>
-      <c r="D50" s="60"/>
+        <v>49517.299327083609</v>
+      </c>
+      <c r="D50" s="66"/>
     </row>
     <row r="51" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="44"/>
       <c r="B51" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="C51" s="59">
+      <c r="C51" s="65">
         <f>SUM(C49:D50)</f>
-        <v>457763.13232416136</v>
-      </c>
-      <c r="D51" s="60"/>
+        <v>430419.60184311139</v>
+      </c>
+      <c r="D51" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="C51:D51"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -8378,11 +8383,6 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="portrait" r:id="rId1"/>

</xml_diff>